<commit_message>
Refine enemy pressure and add hill objective
</commit_message>
<xml_diff>
--- a/docs/design/enemies-arenas-modifiers-balance.xlsx
+++ b/docs/design/enemies-arenas-modifiers-balance.xlsx
@@ -43,6 +43,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -59,7 +60,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-08 18:28</t>
+          <t>2026-05-11 11:05</t>
         </is>
       </c>
     </row>
@@ -84,7 +85,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Patch 13B follow-up</t>
+          <t>Enemy steering / tempo / juice / hill objective pass</t>
         </is>
       </c>
     </row>
@@ -132,7 +133,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bruiser added; crossfire side bias; hot-floor telegraphs; death-pop puddles; stronger swarm waves; generator-safe obstacles; persistent enemy projectiles; layout/modifier debug coverage</t>
+          <t>Feeler steering; arena-wide spawn sampling; faster enemy roster; stronger feedback; capture_the_hill objective added and generator rooms deprioritized</t>
         </is>
       </c>
     </row>
@@ -142,6 +143,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -195,7 +197,7 @@
         <v>30</v>
       </c>
       <c r="C2">
-        <v>108.0</v>
+        <v>145.0</v>
       </c>
       <c r="D2">
         <v>10</v>
@@ -211,7 +213,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Baseline melee chaser with short lunge threat</t>
+          <t>Baseline melee chaser with short lunge threat; 0.10s windup, 1.0s cooldown</t>
         </is>
       </c>
     </row>
@@ -225,7 +227,7 @@
         <v>20</v>
       </c>
       <c r="C3">
-        <v>84.0</v>
+        <v>110.0</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -255,7 +257,7 @@
         <v>40</v>
       </c>
       <c r="C4">
-        <v>88.0</v>
+        <v>125.0</v>
       </c>
       <c r="D4">
         <v>15</v>
@@ -271,7 +273,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Burst melee dash enemy</t>
+          <t>Burst melee dash enemy; 0.20s windup, 1.8s cooldown</t>
         </is>
       </c>
     </row>
@@ -285,7 +287,7 @@
         <v>60</v>
       </c>
       <c r="C5">
-        <v>68.0</v>
+        <v>92.0</v>
       </c>
       <c r="D5">
         <v>20</v>
@@ -301,7 +303,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Slow tank melee; 0.45s windup, 0.15s slam, 1.8s recovery</t>
+          <t>Slow tank melee; 0.30s windup, 0.15s slam, 1.4s recovery, 1.9s cooldown</t>
         </is>
       </c>
     </row>
@@ -315,7 +317,7 @@
         <v>180</v>
       </c>
       <c r="C6">
-        <v>82.0</v>
+        <v>105.0</v>
       </c>
       <c r="D6">
         <v>10</v>
@@ -331,7 +333,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Boss support now cycles chaser, charger, bruiser</t>
+          <t>Boss support now cycles chaser, charger, bruiser; higher baseline pace</t>
         </is>
       </c>
     </row>
@@ -1521,6 +1523,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1642,6 +1645,78 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Feeler steering</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Enemies now probe +/- 30 degrees out to 48px and steer before contact; blocked-time flip remains fallback only</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Separation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nearby enemies repel within 22px with capped force at 35% of move speed so Swarm spreads without overriding pursuit</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Enemy juice pass</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Enemy attack trails, stronger impact/death/explosion particles, heavier hitstop/trauma, and shake ceiling 34 with faster decay 3.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Screen effects default</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Default profile screen-effects setting is now Full so the current combat-feedback pass is visible without manual setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Wave spawn sampling</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Wave/support enemies now sample valid arena positions instead of fixed markers; spawns must avoid players, obstacles, and active objective/interact clutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hill objective</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Capture-the-hill rooms use a sampled control zone plus normal combat-wave pressure; preferred over generator objectives for near-term combat iteration</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Patch 14 arena layout identity pass
</commit_message>
<xml_diff>
--- a/docs/design/enemies-arenas-modifiers-balance.xlsx
+++ b/docs/design/enemies-arenas-modifiers-balance.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -60,7 +60,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-11 11:05</t>
+          <t>2026-05-11 13:51</t>
         </is>
       </c>
     </row>
@@ -85,14 +85,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enemy steering / tempo / juice / hill objective pass</t>
+          <t>Patch 14 layout identity pass</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Core room modifiers</t>
+          <t>Live room modifiers</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -104,36 +104,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Disabled recipe modifiers</t>
+          <t>Active normal layouts</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Armoured, Heavy Patrol, Frenzy, Stampede, Friendly Fire, Darkness, One-Way</t>
+          <t>default, lane, pillars, ring, pockets</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Active obstacle layouts</t>
+          <t>Legacy debug-only layouts</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>pillars, ring, pockets, lane, gauntlet_pockets</t>
+          <t>crossfire, pinch, offset, gauntlet_pockets</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Recipe identities</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Open Swarm, Hold Lanes, Cover Fight, Ring Run, Dead Zone, Pocket Breakthrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Key runtime shifts</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Feeler steering; arena-wide spawn sampling; faster enemy roster; stronger feedback; capture_the_hill objective added and generator rooms deprioritized</t>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>One-layout-per-recipe identities; disabled modifiers removed from encounter data; legacy layouts kept only for builder/debug coverage; pockets recipe remains capture_the_hill</t>
         </is>
       </c>
     </row>
@@ -343,6 +355,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -384,82 +397,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>frenzy</t>
+          <t>hot_floor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Frenzy</t>
+          <t>Hot Floor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>spatial</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>enemy_speed_multiplier=1.35, enemy_fire_interval_multiplier=0.92, spawn_interval_multiplier=0.88</t>
+          <t>hot_floor_zone_interval=7.0, hot_floor_zone_radius=120.0, hot_floor_zone_damage=8, hot_floor_warning_duration=1.5, hot_floor_active_duration=2.5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Enemies move and attack faster. New waves arrive sooner.</t>
+          <t>Telegraphed floor zones ignite in bursts. Move before they flare up.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>armoured</t>
+          <t>death_pop</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Armoured</t>
+          <t>Death Pop</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>disabled</t>
+          <t>spatial</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>enemy_bonus_health=20</t>
+          <t>death_puddle_radius=84.0, death_puddle_tick_damage=6, death_puddle_tick_interval=0.5, death_puddle_warning_duration=0.4, death_puddle_active_duration=2.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Enemies take more punishment before they go down.</t>
+          <t>Enemy deaths leave brief danger puddles. Finish fights in safe spaces.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>hot_floor</t>
+          <t>crossfire</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hot Floor</t>
+          <t>Crossfire</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -468,33 +481,33 @@
         </is>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>spatial</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>hot_floor_zone_interval=7.0, hot_floor_zone_radius=120.0, hot_floor_zone_damage=8, hot_floor_warning_duration=1.5, hot_floor_active_duration=2.5</t>
+          <t>enemy_fire_interval_multiplier=0.82, spawn_interval_multiplier=0.96, spawn_position_bias=sides</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Telegraphed floor zones ignite in bursts. Move before they flare up.</t>
+          <t>Side-biased ranged pressure with faster volleys.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>death_pop</t>
+          <t>swarm</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Death Pop</t>
+          <t>Swarm</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -503,266 +516,21 @@
         </is>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>spatial</t>
+          <t>pressure</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>death_puddle_radius=84.0, death_puddle_tick_damage=6, death_puddle_tick_interval=0.5, death_puddle_warning_duration=0.4, death_puddle_active_duration=2.0</t>
+          <t>spawn_interval_multiplier=0.2, wave_size_bonus=8, enemy_speed_multiplier=0.88, enemy_bonus_health=-10, enemy_contact_damage_bonus=5</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Enemy deaths leave brief danger puddles. Finish fights in safe spaces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>stampede</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Stampede</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>enemy_speed_multiplier=1.18, enemy_contact_damage_bonus=10</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Enemies crash harder on contact and push closer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>crossfire</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Crossfire</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>spatial</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>enemy_fire_interval_multiplier=0.82, spawn_interval_multiplier=0.96, spawn_position_bias=sides</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Ranged enemies pressure the flanks with faster volleys.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>darkness</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Darkness</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>vision_radius=280.0</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Visibility collapses outside the squad. Stay close enough to read the room.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>one_way</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>One-Way</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>spawn_side=left</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Directional spawn-side modifier kept in data only; removed from live encounter rotation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>friendly_fire</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Friendly Fire</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>friendly_fire=True</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Your shots can hit allies. Tight formations become a liability.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>swarm</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Swarm</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>core</t>
-        </is>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>pressure</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>spawn_interval_multiplier=0.2, wave_size_bonus=8, enemy_speed_multiplier=0.88, enemy_bonus_health=-10, enemy_contact_damage_bonus=5</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Very high-pressure horde room modifier: many more enemies, much faster arrivals, each one still slightly weaker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>heavy_patrol</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Heavy Patrol</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="D12">
-        <v>2</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>spawn_interval_multiplier=1.4, enemy_bonus_health=20, enemy_speed_multiplier=0.92</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Fewer waves, but every enemy is tougher. Pick your fights.</t>
+          <t>Larger weaker waves push crowd-control pressure.</t>
         </is>
       </c>
     </row>
@@ -772,6 +540,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -816,187 +585,187 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>open_swarm / chaos_room fallback</t>
+          <t>open_swarm</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Flat readable rectangle</t>
+          <t>Open baseline. No obstacles; broad edge spawning and kite space.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>crossfire</t>
+          <t>lane</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>open-side pressure</t>
+          <t>divider walls</t>
         </is>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>crossfire_lanes fallback</t>
+          <t>hold_lanes</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Open room with side spawn pressure</t>
+          <t>Three broad lanes. Hold fronts and rotate between gaps.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>pinch</t>
+          <t>pillars</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>open pinch</t>
+          <t>circular pillars</t>
         </is>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>hold_the_line fallback</t>
+          <t>cover_fight</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Directional pressure without cover</t>
+          <t>Cover and line-of-sight room. Center stays open for loot.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>offset</t>
+          <t>ring</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>open asymmetry</t>
+          <t>circular loop pillars</t>
         </is>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>open_swarm</t>
+          <t>ring_run / dead_zone</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Slightly skewed open room</t>
+          <t>Outer loop with cut-through route decisions.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>pillars</t>
+          <t>pockets</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>circular pillars</t>
+          <t>circular pillar pairs</t>
         </is>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>pillar_skirmish / dead_zone_ring</t>
+          <t>pocket_breakthrough</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Center reserved for loot; cover-focused skirmish</t>
+          <t>Push into defended pockets and hold the contested zone.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ring</t>
+          <t>crossfire</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>tight pillar loop</t>
+          <t>legacy open-side pressure</t>
         </is>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ring_run / dead_zone_ring</t>
+          <t>debug only</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Risk-reward center cuts and loop kiting</t>
+          <t>Legacy layout kept only for builder/debug regression coverage.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pockets</t>
+          <t>pinch</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>paired pillar pockets</t>
+          <t>legacy open pinch</t>
         </is>
       </c>
       <c r="C8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>pocket_breakthrough</t>
+          <t>debug only</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Objective pockets open toward center retreat lane; generator slots are sanitized away from blockers</t>
+          <t>Legacy layout kept only for builder/debug regression coverage.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>lane</t>
+          <t>offset</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>broad horizontal divider walls</t>
+          <t>legacy open asymmetry</t>
         </is>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>hold_the_line / crossfire_lanes</t>
+          <t>debug only</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Three combat lanes with wide side rotation gaps; revive path and generators must stay reachable</t>
+          <t>Legacy layout kept only for builder/debug regression coverage.</t>
         </is>
       </c>
     </row>
@@ -1008,7 +777,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>generator gauntlet</t>
+          <t>legacy generator pockets</t>
         </is>
       </c>
       <c r="C10">
@@ -1016,12 +785,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>generator default</t>
+          <t>debug only</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Authored generator-room layout</t>
+          <t>Legacy generator-focused layout kept only for builder/debug regression coverage.</t>
         </is>
       </c>
     </row>
@@ -1033,7 +802,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>boss arena</t>
+          <t>boss staging walls</t>
         </is>
       </c>
       <c r="C11">
@@ -1046,7 +815,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Boss endpoint with no modifier recipe</t>
+          <t>Boss-only layout. Not used by normal combat recipes.</t>
         </is>
       </c>
     </row>
@@ -1056,6 +825,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:I7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1112,7 +882,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>default, offset</t>
+          <t>default</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1130,11 +900,9 @@
           <t>survive</t>
         </is>
       </c>
-      <c r="F2"/>
       <c r="G2">
         <v>2</v>
       </c>
-      <c r="H2"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Readable horde room. Mow down many weak enemies.</t>
@@ -1144,17 +912,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>hold_the_line</t>
+          <t>hold_lanes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>lane, pinch</t>
+          <t>lane</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t/>
+          <t>, crossfire</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1167,34 +935,31 @@
           <t>survive</t>
         </is>
       </c>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Defend against a directional push through geometry and enemy mix, without a side-spawn modifier.</t>
+          <t>Hold fronts and rotate between lanes.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>crossfire_lanes</t>
+          <t>cover_fight</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>lane, crossfire</t>
+          <t>pillars</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>crossfire</t>
+          <t>crossfire, death_pop</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>spitter_chaser</t>
+          <t>spitter_bruiser</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1202,34 +967,31 @@
           <t>survive</t>
         </is>
       </c>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Dodge ranged side pressure while clearing spitters.</t>
+          <t>Use cover and clear ranged pressure around pillars.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pillar_skirmish</t>
+          <t>ring_run</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>pillars</t>
+          <t>ring</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>crossfire, death_pop</t>
+          <t>hot_floor, swarm</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>spitter_bruiser</t>
+          <t>chaser_charger</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1237,19 +999,19 @@
           <t>survive</t>
         </is>
       </c>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
+      <c r="F5">
+        <v>2.2</v>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use cover, clear ranged threats, manage blockers.</t>
+          <t>Continuous looping movement with route decisions.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ring_run</t>
+          <t>dead_zone</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1259,12 +1021,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>hot_floor, swarm</t>
+          <t>death_pop</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>chaser_charger</t>
+          <t>bruiser_mix</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1272,125 +1034,36 @@
           <t>survive</t>
         </is>
       </c>
-      <c r="F6">
-        <v>2.2</v>
-      </c>
-      <c r="G6"/>
-      <c r="H6"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Continuous looping movement.</t>
+          <t>Kill enemies in safe spaces, avoid death zones.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dead_zone_ring</t>
+          <t>pocket_breakthrough</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ring, pillars</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>death_pop</t>
+          <t>pockets</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bruiser_mix</t>
+          <t>bruiser_spitter_chaser</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>survive</t>
-        </is>
-      </c>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
+          <t>capture_the_hill</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Kill enemies in safe places, avoid death zones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>pocket_breakthrough</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>pockets</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>bruiser_spitter_chaser</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>destroy_generators</t>
-        </is>
-      </c>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Push into defended pockets and destroy objectives without directional spawn-side gimmicks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>chaos_room</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>default, ring</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>hot_floor, death_pop</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>survive</t>
-        </is>
-      </c>
-      <c r="F9">
-        <v>1.8</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
-        <v>4.0</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Late-run spectacle.</t>
+          <t>Push into defended pockets and hold the contested objective.</t>
         </is>
       </c>
     </row>
@@ -1400,6 +1073,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1419,7 +1093,6 @@
           <t>default</t>
         </is>
       </c>
-      <c r="B2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1448,72 +1121,36 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>spitter_chaser</t>
+          <t>spitter_bruiser</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4, 3, 0, 0</t>
+          <t>2, 3, 0, 3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>spitter_bruiser</t>
+          <t>bruiser_spitter_chaser</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2, 3, 0, 3</t>
+          <t>3, 2, 1, 3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>chaser_charger_bruiser</t>
+          <t>bruiser_mix</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3, 0, 3, 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>bruiser_spitter_chaser</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3, 2, 1, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>bruiser_mix</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
           <t>2, 0, 2, 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>3, 2, 2, 2</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1545,175 +1182,127 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Never place obstacles on the arena center; loot/interact flow must stay clear</t>
+          <t>Never place obstacles on the arena center; loot/interact flow must stay clear.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Crossfire rework</t>
+          <t>Layout identity rule</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Side-biased spitter spawns plus faster volleys; spatial identity first</t>
+          <t>Each normal layout must force a behavior Open does not.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hot Floor rework</t>
+          <t>Recipe selection</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2-3 telegraphed zones per batch; warning before active damage</t>
+          <t>Anti-repeat excludes the last 2 recipe IDs when possible.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Death Pop rework</t>
+          <t>Modifier pairing</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enemy deaths leave temporary puddles with warning, not instant burst damage</t>
+          <t>Recipes are the pairing rules; no separate global modifier-pairing table is needed.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Recipe selection</t>
+          <t>Legacy layouts</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Anti-repeat excludes the last 2 recipe IDs when possible</t>
+          <t>crossfire, pinch, offset, and gauntlet_pockets stay builder-only for regression testing.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Debug testing</t>
+          <t>Crossfire role</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Debug single-room mode can now test modifiers and layouts independently, including pillars/ring/pockets/lane</t>
+          <t>Crossfire is modifier-only in normal recipes and uses side-biased spitter spawns plus faster volleys.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Generator compatibility</t>
+          <t>Pockets role</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Generator rooms reject directional spawn-side modifiers and sanitize generator slots away from obstacle geometry</t>
+          <t>Pocket Breakthrough uses capture_the_hill so the layout plays as a push-and-hold room.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Swarm tuning</t>
+          <t>Generator compatibility</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Swarm now owns a 200% spawn-rate increase plus large modifier wave-size bonus</t>
+          <t>Generator rooms still sanitize target slots away from obstacle geometry.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Enemy projectiles</t>
+          <t>Swarm tuning</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enemy projectiles now persist until they hit a wall, obstacle, or target instead of timing out mid-flight</t>
+          <t>Swarm owns a 200% spawn-rate increase plus a large modifier wave-size bonus.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Feeler steering</t>
+          <t>Ring intent</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Enemies now probe +/- 30 degrees out to 48px and steer before contact; blocked-time flip remains fallback only</t>
+          <t>Ring should force looping movement and cut-through decisions rather than read like another open room.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Separation</t>
+          <t>Builder testing</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Nearby enemies repel within 22px with capped force at 35% of move speed so Swarm spreads without overriding pursuit</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Enemy juice pass</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Enemy attack trails, stronger impact/death/explosion particles, heavier hitstop/trauma, and shake ceiling 34 with faster decay 3.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Screen effects default</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Default profile screen-effects setting is now Full so the current combat-feedback pass is visible without manual setup</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Wave spawn sampling</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Wave/support enemies now sample valid arena positions instead of fixed markers; spawns must avoid players, obstacles, and active objective/interact clutter</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Hill objective</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Capture-the-hill rooms use a sampled control zone plus normal combat-wave pressure; preferred over generator objectives for near-term combat iteration</t>
+          <t>Encounter Builder should cover each live layout with approved modifiers plus legacy-layout regression launches.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement roadmap runtime systems and sustain tuning
</commit_message>
<xml_diff>
--- a/docs/design/enemies-arenas-modifiers-balance.xlsx
+++ b/docs/design/enemies-arenas-modifiers-balance.xlsx
@@ -64,7 +64,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OUTDATED: This workbook reflects an older encounter/layout/modifier branch state and is not the current runtime source of truth. See docs/development/current-state.md and docs/design/roadmap.md.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>